<commit_message>
Relatório dos dias trabalhados da ANA CELIA no Centro em agosto
Dia a dia das vendas registradas no código 131, com pedidos, itens,
venda bruta e líquida, comissão e o horário da primeira e da última
venda, mais o cálculo das diárias. A aba FOLGUISTAS do relatório do
Centro já vem com os 12 dias apurados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -7995,7 +7995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8108,7 +8108,9 @@
       <c r="C6" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="8" t="n">
+        <v>12</v>
+      </c>
       <c r="E6" s="56">
         <f>C6*D6</f>
         <v/>
@@ -8167,24 +8169,32 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Comissão e incentivos vêm do relatório do InovaFarma (códigos 51 e 131) — CONFIRMAR se o folguista recebe esses valores além da diária; se não receber, zerar as colunas.</t>
+          <t>ANA CELIA: 12 dias com venda registrada em agosto/2026 (quartas, sextas e domingos) — ver o relatório ANA_CELIA_DIAS_TRABALHADOS_AGOSTO_2026.xlsx. Conferir com a escala.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>Comissão e incentivos vêm do relatório do InovaFarma (códigos 51 e 131) — CONFIRMAR se o folguista recebe esses valores além da diária; se não receber, zerar as colunas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>Estes valores não entram no holerite: são pagamento de prestação de serviço, para baixa no contas a pagar.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:H6"/>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Relatório dos dias trabalhados do SERGIO e generalização do script
Mesmo levantamento feito para a ANA CELIA, agora para o SERGIO (código
51). O script passa a receber o folguista como argumento e destaca dias
com uma única venda simbólica, que provavelmente não valem diária —
01/08 e 26/08 no caso dele.

A aba FOLGUISTAS do Centro já vem com 12 dias da ANA CELIA e 7 do
SERGIO, com a ressalva sobre os dois dias a conferir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -7995,7 +7995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8078,7 +8078,9 @@
       <c r="C5" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="8" t="n">
+        <v>7</v>
+      </c>
       <c r="E5" s="56">
         <f>C5*D5</f>
         <v/>
@@ -8169,33 +8171,49 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>ANA CELIA: 12 dias com venda registrada em agosto/2026 (quartas, sextas e domingos) — ver o relatório ANA_CELIA_DIAS_TRABALHADOS_AGOSTO_2026.xlsx. Conferir com a escala.</t>
+          <t>ANA CELIA: 12 dias com venda registrada em agosto/2026 (quartas, sextas e domingos).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Comissão e incentivos vêm do relatório do InovaFarma (códigos 51 e 131) — CONFIRMAR se o folguista recebe esses valores além da diária; se não receber, zerar as colunas.</t>
+          <t>SERGIO: 7 dias com venda registrada, sendo 5 com movimento efetivo — 01/08 e 26/08 tiveram uma única venda simbólica no código dele. Ajustar a quantidade se esses dois dias não valerem diária.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Detalhe dia a dia nos relatórios ANA_CELIA_ e SERGIO_DIAS_TRABALHADOS_AGOSTO_2026.xlsx. Conferir com a escala da loja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Comissão e incentivos vêm do relatório do InovaFarma (códigos 51 e 131) — CONFIRMAR se o folguista recebe esses valores além da diária; se não receber, zerar as colunas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
           <t>Estes valores não entram no holerite: são pagamento de prestação de serviço, para baixa no contas a pagar.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:H6"/>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Corrigir as horas extras do INIURLE para 16 h a 50% e 24 h a 100%
As 40 h de agosto eram 16 h a 50% (R$ 176,84) e 24 h a 100%
(R$ 353,67), somando R$ 530,51 no lugar de R$ 442,09. Novo tipo de
ocorrência HE100 na aba de ponto e novo parâmetro do adicional de 100%.

O holerite emitido pela Betel saiu com 40 h a 50%; a diferença aparece
na conferência e fica registrada como pendência para refazer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1315,84 +1315,99 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Adicional noturno</t>
+          <t>Adicional de hora extra 100%</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>20% sobre a hora normal, nas horas entre 22h e 5h.</t>
+          <t>100% sobre a hora normal (hora extra = salário-hora × 2).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Dias do mês para o salário-dia</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>30</v>
+          <t>Adicional noturno</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>0.2</v>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Salário-dia = salário base ÷ 30. Usado no feriado trabalhado.</t>
+          <t>20% sobre a hora normal, nas horas entre 22h e 5h.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
+          <t>Dias do mês para o salário-dia</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Salário-dia = salário base ÷ 30. Usado no feriado trabalhado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
           <t>Multiplicador da comissão</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B21" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>1 = paga o valor apurado no InovaFarma, sem multiplicador.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>INSS / IRRF</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>INSS</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>a calcular</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Calculado pela contabilidade sobre o total de proventos (tabela progressiva vigente).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
+          <t>INSS</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>a calcular</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Calculado pela contabilidade sobre o total de proventos (tabela progressiva vigente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
           <t>IRRF</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>a calcular</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Calculado pela contabilidade após dedução do INSS e dependentes.</t>
         </is>
@@ -1403,7 +1418,7 @@
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -2114,19 +2129,19 @@
         <v>0</v>
       </c>
       <c r="C9" s="34">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F6*PARÂMETROS!$B$20,2)</f>
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F6*PARÂMETROS!$B$21,2)</f>
         <v/>
       </c>
       <c r="D9" s="34">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F7*PARÂMETROS!$B$20,2)</f>
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F7*PARÂMETROS!$B$21,2)</f>
         <v/>
       </c>
       <c r="E9" s="34">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F8*PARÂMETROS!$B$20,2)</f>
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F8*PARÂMETROS!$B$21,2)</f>
         <v/>
       </c>
       <c r="F9" s="34">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F9*PARÂMETROS!$B$20,2)</f>
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F9*PARÂMETROS!$B$21,2)</f>
         <v/>
       </c>
       <c r="G9" s="34" t="n">

</xml_diff>

<commit_message>
Registrar que o PEDRO é da empresa matriz
O PEDRO é registrado na Farmácia Tropical Ltda (matriz). A pendência de
agosto deixa de ser "descobrir a empresa" e passa a ser pedir à Betel o
holerite de agosto dele, que não veio no arquivo. Capas, resumos e a
passagem de trabalho atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -845,7 +845,7 @@
       <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>GENECIR: férias de 01 a 30/08/2026, já pagas em recibo próprio — salário zerado neste holerite; confirmar o dia 31/08.</t>
+          <t>PEDRO é registrado na empresa matriz (Farmácia Tropical Ltda).</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       <c r="A24" s="4" t="inlineStr"/>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>SERGIO e ANA CELIA são folguistas (diária de R$ 150,00 e R$ 100,00) — ficam na aba FOLGUISTAS, para o contas a pagar, fora do holerite.</t>
+          <t>GENECIR: férias de 01 a 30/08/2026, já pagas em recibo próprio — salário zerado neste holerite; confirmar o dia 31/08.</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       <c r="A25" s="4" t="inlineStr"/>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>GILSON, UILLIAN e FABIANA não recebem comissão pela loja Centro.</t>
+          <t>SERGIO e ANA CELIA são folguistas (diária de R$ 150,00 e R$ 100,00) — ficam na aba FOLGUISTAS, para o contas a pagar, fora do holerite.</t>
         </is>
       </c>
     </row>
@@ -869,26 +869,22 @@
       <c r="A26" s="4" t="inlineStr"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
+          <t>GILSON, UILLIAN e FABIANA não recebem comissão pela loja Centro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
           <t>SARA: o saldo dela na loja Centro foi somado à folha do Arraial.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>PENDÊNCIAS — CONFIRMAR ANTES DE ENVIAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Horas extras, adicional noturno e feriados trabalhados de agosto — lançar na aba PONTO AGO.26.</t>
         </is>
       </c>
     </row>
@@ -900,7 +896,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Prêmio cota geral e prêmio pré-vencidos, conforme a tabela de metas da loja.</t>
+          <t>Horas extras, adicional noturno e feriados trabalhados de agosto — lançar na aba PONTO AGO.26.</t>
         </is>
       </c>
     </row>
@@ -912,7 +908,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Vales adiantados, convênio e faltas de agosto.</t>
+          <t>Prêmio cota geral e prêmio pré-vencidos, conforme a tabela de metas da loja.</t>
         </is>
       </c>
     </row>
@@ -924,7 +920,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Férias, afastamentos e admissões que mudem o salário do mês.</t>
+          <t>Vales adiantados, convênio e faltas de agosto.</t>
         </is>
       </c>
     </row>
@@ -936,7 +932,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>PEDRO não aparece no holerite de agosto emitido pela Betel para esta loja — verificar em qual empresa ele foi lançado.</t>
+          <t>Férias, afastamentos e admissões que mudem o salário do mês.</t>
         </is>
       </c>
     </row>
@@ -948,7 +944,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>GENECIR: a comissão de R$ 0,62 não entrou no holerite (ele passou o mês de férias) — conferir se vale lançar.</t>
+          <t>PEDRO é registrado na matriz (Farmácia Tropical Ltda), mas o holerite de agosto dele NÃO veio no arquivo da Betel — pedir à Betel o holerite de agosto (salário R$ 1.621,00, sem comissão).</t>
         </is>
       </c>
     </row>
@@ -960,7 +956,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>GENECIR: as férias vão até 30/08 e o mês tem 31 dias — confirmar se o dia 31/08 foi trabalhado e lançar o salário desse dia (R$ 1.621,00 ÷ 30 = R$ 54,03).</t>
+          <t>GENECIR: a comissão de R$ 0,62 não entrou no holerite (ele passou o mês de férias) — conferir se vale lançar.</t>
         </is>
       </c>
     </row>
@@ -972,7 +968,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Preencher a quantidade de diárias de SERGIO e ANA CELIA na aba FOLGUISTAS.</t>
+          <t>GENECIR: as férias vão até 30/08 e o mês tem 31 dias — confirmar se o dia 31/08 foi trabalhado e lançar o salário desse dia (R$ 1.621,00 ÷ 30 = R$ 54,03).</t>
         </is>
       </c>
     </row>
@@ -984,37 +980,41 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
+          <t>Preencher a quantidade de diárias de SERGIO e ANA CELIA na aba FOLGUISTAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
           <t>Confirmar se os folguistas recebem a comissão apurada no código deles (SERGIO R$ 128,80 e ANA CELIA R$ 83,56) além da diária.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO TÉCNICA</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="17" customHeight="1">
-      <c r="A38" s="4" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>As células de total e de cálculo são fórmulas. Ao abrir no Excel ou no Google Planilhas elas aparecem calculadas; em visualizadores simples podem aparecer em branco até o arquivo ser aberto.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>ABAS DO ARQUIVO</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="17" customHeight="1">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
+          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       <c r="A42" s="4" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
+          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       <c r="A43" s="4" t="inlineStr"/>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>JULHO.26 REVISADO — a folha de julho (CENTRO 05JULHO) reorganizada e conferida.</t>
+          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       <c r="A45" s="4" t="inlineStr"/>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
+          <t>JULHO.26 REVISADO — a folha de julho (CENTRO 05JULHO) reorganizada e conferida.</t>
         </is>
       </c>
     </row>
@@ -1062,13 +1062,21 @@
       <c r="A46" s="4" t="inlineStr"/>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
+          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="17" customHeight="1">
       <c r="A47" s="4" t="inlineStr"/>
       <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="17" customHeight="1">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>FOLGUISTAS — diárias de SERGIO e ANA CELIA para o contas a pagar (fora do holerite).</t>
         </is>
@@ -1079,12 +1087,12 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A38:B38"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>